<commit_message>
Fill criteria for 8 of 9 states from retrieved state and MCO documents (DE, KS, MI, NC, PA, RI, TN, UT); reclassify UT and RI as more restrictive; only SC remains not documented
</commit_message>
<xml_diff>
--- a/outputs/state_coverage_summary.xlsx
+++ b/outputs/state_coverage_summary.xlsx
@@ -992,7 +992,7 @@
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>more_restrictive</t>
+          <t>more_restrictive (BMI 30 with risk-factor logic, three-month low-calorie diet trial; MCO policy and SPA)</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
@@ -1400,7 +1400,7 @@
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>more_restrictive</t>
+          <t>more_restrictive (BMI-40 high-cost tier, waived for Zepbound 4/1/24 and Wegovy 6/1/25; lifestyle required)</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
@@ -1736,7 +1736,7 @@
       </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
-          <t>more_restrictive</t>
+          <t>more_restrictive (appropriateness PA 2022 to 2025; BMI-40 morbid-obesity criteria from 1/1/2026)</t>
         </is>
       </c>
       <c r="L23" s="2" t="inlineStr">
@@ -2072,7 +2072,7 @@
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
-          <t>more_restrictive (clinical criteria apply to all drugs in class)</t>
+          <t>fda_label</t>
         </is>
       </c>
       <c r="L28" s="2" t="inlineStr">
@@ -2648,7 +2648,7 @@
       </c>
       <c r="K39" s="2" t="inlineStr">
         <is>
-          <t>fda_label (per Klebanoff); criteria not in documents in hand</t>
+          <t>more_restrictive (MCO form; requires concurrent diabetes or antidiabetic use in past 120 days before a preferred GLP-1)</t>
         </is>
       </c>
       <c r="L39" s="2" t="inlineStr">
@@ -2720,7 +2720,7 @@
       </c>
       <c r="K40" s="2" t="inlineStr">
         <is>
-          <t>not_documented (clinical PA for entire class, manual PA)</t>
+          <t>more_restrictive (6-month supervised weight-management program before drug therapy; MCO policy)</t>
         </is>
       </c>
       <c r="L40" s="2" t="inlineStr">
@@ -2912,7 +2912,7 @@
       </c>
       <c r="K43" s="2" t="inlineStr">
         <is>
-          <t>not_documented (PA, QL flagged; criteria in Optum Rx TennCare criteria document, not in folder)</t>
+          <t>fda_label</t>
         </is>
       </c>
       <c r="L43" s="2" t="inlineStr">
@@ -3032,7 +3032,7 @@
       </c>
       <c r="K45" s="2" t="inlineStr">
         <is>
-          <t>not_documented (PA criteria document on Utah Medicaid PA page, not in folder)</t>
+          <t>more_restrictive (6 months of dietitian-supervised lifestyle trials required)</t>
         </is>
       </c>
       <c r="L45" s="2" t="inlineStr">
@@ -3612,7 +3612,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>more_restrictive</t>
+          <t>more_restrictive (BMI 30 with risk-factor logic, three-month low-calorie diet trial; MCO policy and SPA)</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -3654,7 +3654,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>more_restrictive</t>
+          <t>more_restrictive (BMI 30 with risk-factor logic, three-month low-calorie diet trial; MCO policy and SPA)</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -3696,7 +3696,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>more_restrictive</t>
+          <t>more_restrictive (BMI 30 with risk-factor logic, three-month low-calorie diet trial; MCO policy and SPA)</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -3738,12 +3738,12 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>more_restrictive</t>
+          <t>more_restrictive (BMI-40 high-cost tier, waived for Zepbound 4/1/24 and Wegovy 6/1/25; lifestyle required)</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>9/6/2024</t>
+          <t>8/19/2026</t>
         </is>
       </c>
     </row>
@@ -3780,12 +3780,12 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>more_restrictive</t>
+          <t>more_restrictive (BMI-40 high-cost tier, waived for Zepbound 4/1/24 and Wegovy 6/1/25; lifestyle required)</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>9/6/2024</t>
+          <t>8/19/2026</t>
         </is>
       </c>
     </row>
@@ -3822,12 +3822,12 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>more_restrictive</t>
+          <t>more_restrictive (BMI-40 high-cost tier, waived for Zepbound 4/1/24 and Wegovy 6/1/25; lifestyle required)</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>9/6/2024</t>
+          <t>8/19/2026</t>
         </is>
       </c>
     </row>
@@ -3990,12 +3990,12 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>more_restrictive</t>
+          <t>more_restrictive (appropriateness PA 2022 to 2025; BMI-40 morbid-obesity criteria from 1/1/2026)</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>8/1/2025</t>
+          <t>1/1/2026</t>
         </is>
       </c>
     </row>
@@ -4032,12 +4032,12 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>more_restrictive</t>
+          <t>more_restrictive (appropriateness PA 2022 to 2025; BMI-40 morbid-obesity criteria from 1/1/2026)</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>8/1/2025</t>
+          <t>1/1/2026</t>
         </is>
       </c>
     </row>
@@ -4074,12 +4074,12 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>more_restrictive</t>
+          <t>more_restrictive (appropriateness PA 2022 to 2025; BMI-40 morbid-obesity criteria from 1/1/2026)</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>8/1/2025</t>
+          <t>1/1/2026</t>
         </is>
       </c>
     </row>
@@ -4368,12 +4368,12 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>more_restrictive (clinical criteria apply to all drugs in class)</t>
+          <t>fda_label</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>8/1/2024</t>
+          <t>7/1/2024</t>
         </is>
       </c>
     </row>
@@ -4410,12 +4410,12 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>more_restrictive (clinical criteria apply to all drugs in class)</t>
+          <t>fda_label</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>8/1/2024</t>
+          <t>7/1/2024</t>
         </is>
       </c>
     </row>
@@ -4452,12 +4452,12 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>more_restrictive (clinical criteria apply to all drugs in class)</t>
+          <t>fda_label</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>8/1/2024</t>
+          <t>7/1/2024</t>
         </is>
       </c>
     </row>
@@ -4620,12 +4620,12 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>fda_label (per Klebanoff); criteria not in documents in hand</t>
+          <t>more_restrictive (MCO form; requires concurrent diabetes or antidiabetic use in past 120 days before a preferred GLP-1)</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>7/7/2025</t>
+          <t>1/6/2025</t>
         </is>
       </c>
     </row>
@@ -4662,12 +4662,12 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>fda_label (per Klebanoff); criteria not in documents in hand</t>
+          <t>more_restrictive (MCO form; requires concurrent diabetes or antidiabetic use in past 120 days before a preferred GLP-1)</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>7/7/2025</t>
+          <t>1/6/2025</t>
         </is>
       </c>
     </row>
@@ -4704,12 +4704,12 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>fda_label (per Klebanoff); criteria not in documents in hand</t>
+          <t>more_restrictive (MCO form; requires concurrent diabetes or antidiabetic use in past 120 days before a preferred GLP-1)</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>7/7/2025</t>
+          <t>1/6/2025</t>
         </is>
       </c>
     </row>
@@ -4746,12 +4746,12 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>not_documented (clinical PA for entire class, manual PA)</t>
+          <t>more_restrictive (6-month supervised weight-management program before drug therapy; MCO policy)</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>5/21/2024</t>
+          <t>5/15/2024</t>
         </is>
       </c>
     </row>
@@ -4788,12 +4788,12 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>not_documented (clinical PA for entire class, manual PA)</t>
+          <t>more_restrictive (6-month supervised weight-management program before drug therapy; MCO policy)</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>5/21/2024</t>
+          <t>5/15/2024</t>
         </is>
       </c>
     </row>
@@ -4830,12 +4830,12 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>not_documented (clinical PA for entire class, manual PA)</t>
+          <t>more_restrictive (6-month supervised weight-management program before drug therapy; MCO policy)</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>5/21/2024</t>
+          <t>5/15/2024</t>
         </is>
       </c>
     </row>
@@ -4948,7 +4948,7 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>not_documented (PA, QL flagged; criteria in Optum Rx TennCare criteria document, not in folder)</t>
+          <t>fda_label</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
@@ -4990,7 +4990,7 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>not_documented (PA, QL flagged; criteria in Optum Rx TennCare criteria document, not in folder)</t>
+          <t>fda_label</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
@@ -5032,7 +5032,7 @@
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>not_documented (PA, QL flagged; criteria in Optum Rx TennCare criteria document, not in folder)</t>
+          <t>fda_label</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
@@ -5074,7 +5074,7 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>not_documented (PA criteria document on Utah Medicaid PA page, not in folder)</t>
+          <t>more_restrictive (6 months of dietitian-supervised lifestyle trials required)</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
@@ -5116,7 +5116,7 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>not_documented (PA criteria document on Utah Medicaid PA page, not in folder)</t>
+          <t>more_restrictive (6 months of dietitian-supervised lifestyle trials required)</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
@@ -5158,7 +5158,7 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>not_documented (PA criteria document on Utah Medicaid PA page, not in folder)</t>
+          <t>more_restrictive (6 months of dietitian-supervised lifestyle trials required)</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
@@ -6554,37 +6554,37 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>more_restrictive</t>
+          <t>more_restrictive (BMI 30 with risk-factor logic, three-month low-calorie diet trial; MCO policy and SPA)</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>SPA DE-24-0010: "The State will cover drugs indicated for the treatment of obesity to address weight loss with co-morbid conditions with prior authorization" (comorbidity required; BMI threshold not stated in documents in hand)</t>
+          <t>BMI above 30 with no risk factors, or above 27 with at least one very-high-risk factor (type 2 diabetes, coronary heart disease, atherosclerotic disease, sleep apnea), or waist circumference above 102 cm (men) or 88 cm (women) with a very-high-risk factor. SPA DE-24-0010: coverage for obesity with co-morbid conditions and PA</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Not documented</t>
+          <t>No separate adolescent BMI threshold (Saxenda age 18+; Xenical 12+)</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>2025 PDL: two preferred products required before a non-preferred product (Saxenda non-preferred; Wegovy, Zepbound preferred)</t>
+          <t>Documented failure of at least a three-month low-calorie diet trial and increased physical activity</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Not documented</t>
+          <t>18 (Saxenda)</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Not documented (evidence file: QL No)</t>
+          <t>Initial approval 3 months; 3-month check (at least 4 lb first month, 1 lb/month next two); 6-month renewal at 5% loss; further renewal at 10% loss and maintenance</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Statewide PDL; MCO policy DE.PMN.50 (Delaware First Health) cited by Khanna et al.</t>
+          <t>Delaware First Health (Centene MCO) policy DE.PMN.50; SPA DE-24-0010 sets the state coverage floor</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
@@ -6594,7 +6594,7 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>SPA DE-24-0010 approved with effective date August 1, 2024; Delaware Medicaid PDL 2025 Obesity Treatment Agents (p. 44); 23 DE Reg 464 (2019)</t>
+          <t>SPA DE-24-0010 (effective 8/1/2024); Delaware First Health Clinical Policy DE.PMN.50 Anti-Obesity Medications, effective 01.23, https://delawarefirsthealth.com/content/dam/centene/delaware/Policies/DrugPolicies/DE.PMN.50%20Anti-Obesity%20Medications%2001.23.pdf</t>
         </is>
       </c>
     </row>
@@ -6606,47 +6606,47 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>more_restrictive</t>
+          <t>more_restrictive (BMI-40 high-cost tier, waived for Zepbound 4/1/24 and Wegovy 6/1/25; lifestyle required)</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Zepbound (preferred): BMI 30 or higher, or 27 or higher with at least one weight-related comorbidity; Saxenda or Wegovy (non-preferred): BMI 40 or higher; Wegovy with BMI 27 or higher only for established CVD without diabetes (MCO bulletin, Sept 2024; KDHE PA form rev. 08/2026 gives adults BMI 40 or higher for non-preferred)</t>
+          <t>Age 18 or older: BMI 30 or higher, or 27 or higher with a weight-related comorbidity (Table 2). High-cost tier (Table 4): BMI 40 or higher; Wegovy also BMI 27 or higher with established CVD and no diabetes. The Table 4 BMI-40 requirement does not apply to Zepbound (from 4/1/24) or Wegovy (from 6/1/25)</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>KDHE form (rev. 08/2026): adolescents 12 to 17, BMI 140% of the 95th percentile or 40 or higher</t>
+          <t>Ages 12 to 17: BMI at or above the 95th percentile (Table 3); high-cost tier requires 140% of the 95th percentile or 40 or higher</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Must try and fail Zepbound before other GLP-1 agents; lifestyle interventions required (not for Zepbound); one-year wait after a failed GLP-1</t>
+          <t>Preferred PDL agent required if applicable; at least 3 months of documented lifestyle modification; type 2 diabetes patients must use the diabetes formulation; 1-year wait after a failed Table 4 agent (not for Zepbound or Wegovy)</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>12 (adolescent criteria)</t>
+          <t>12 (Saxenda, Wegovy 2.4 mg); 18 (Zepbound, Foundayo, Wegovy HD)</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Dosing limits per FDA label on PA</t>
+          <t>Initial 28 weeks (Zepbound, Wegovy) or 8 weeks (Table 4 agents); renewal 6 months then 12 months; non-Table-4 adults must lose 5% at 12 weeks or 10% at 28 weeks; dosing per Table 1</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>KDHE statewide PDL applies to KanCare MCOs; criteria quoted from Sunflower Health Plan bulletin SHPBN-2024-036</t>
+          <t>KDHE statewide criteria (apply to KanCare MCOs)</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>9/6/2024</t>
+          <t>8/19/2026</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Sunflower Health Plan bulletin SHPBN-2024-036 (September 6, 2024), https://www.sunflowerhealthplan.com/newsroom/shpbn-2024-036.html; KDHE Anti-Obesity Medications PA form (rev. 08/2026); KMAP Bulletin 24071 (April 17, 2024)</t>
+          <t>KDHE Criteria for Prior Authorization, Anti-Obesity Medications (AOMs), last reviewed 8/19/2026 (prior version 1/17/2024), https://www.kdhe.ks.gov/DocumentCenter/View/407/Anti-Obesity-Medications-PDF; also covers Foundayo (orforglipron)</t>
         </is>
       </c>
     </row>
@@ -6710,32 +6710,32 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>more_restrictive</t>
+          <t>more_restrictive (appropriateness PA 2022 to 2025; BMI-40 morbid-obesity criteria from 1/1/2026)</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Not in documents in hand (criteria are in the MDHHS Common Formulary PA criteria document linked in RA notes); DUR Board minutes: all agents "preferred with clinical prior authorization (PA) for appropriateness"</t>
+          <t>2022 to 2025: clinical PA for appropriateness (DUR Board); specific BMI not in the 2024 Common Formulary. From 1/1/2026: BMI classified as morbidly obese (baseline 40 or higher), framed as averting bariatric surgery</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Not documented (Common Formulary marks AGE PA on Saxenda, Wegovy, Zepbound)</t>
+          <t>From 1/1/2026: BMI classified as morbidly obese per CDC growth charts for age and sex</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Not documented</t>
+          <t>From 1/1/2026: trial and failure or intolerance to all five preferred agent types; documented failure of all other clinically appropriate weight-loss interventions; one weight-loss drug in class at a time; no concurrent DPP-4 inhibitor</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>AGE PA flag (threshold not in documents in hand)</t>
+          <t>12 (Saxenda, Wegovy); 18 (Zepbound)</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Quantity limits apply (2025 PDL footnote 2; MIRx quantity limits document)</t>
+          <t>Saxenda 5 pens per 30 days; Wegovy and Zepbound 4 pens per 28 days; initial 6 months, renewal 6 months; renewal requires 5% weight loss (adults) or maintained/improved BMI percentile (adolescents)</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -6745,12 +6745,12 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>8/1/2025</t>
+          <t>1/1/2026</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>MDHHS DUR Board minutes September 5, 2023; Medicaid Health Plan Common Formulary 11/1/2024; Michigan Single PDL effective 08/01/2025 (p. 39)</t>
+          <t>MDHHS DUR Board minutes September 5, 2023 (appropriateness PA from 2/1/2022); MIRx Single PDL 1.1.2026 anti-obesity GLP-1 criteria, https://mi.primetherapeutics.com/provider/external/medicaid/mi/doc/en-us/MIRx_Miscellaneous_Anti-Obesity_Agents_NonPreferred_GLP1s.pdf</t>
         </is>
       </c>
     </row>
@@ -6918,47 +6918,47 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>more_restrictive (clinical criteria apply to all drugs in class)</t>
+          <t>fda_label</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Not in documents in hand for the August 2024 weight-management criteria (the PA form in the folder is the post-October-2025 version for cardioprotection, NASH and sleep apnea)</t>
+          <t>Age 18 or older: BMI 30 or higher, or 27 or higher with at least one weight-related comorbidity (hypertension, type 2 diabetes, etc.); age 45 or older with BMI 27 or higher and established CVD (Wegovy cardioprotection)</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Not documented</t>
+          <t>Ages 12 to 17: BMI at or above the 95th percentile for age and sex, or at or above the 85th percentile with a comorbidity</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Saxenda and Zepbound non-preferred (August 2024 PDL); Wegovy preferred</t>
+          <t>Saxenda and Zepbound non-preferred (require failed preferred drug); Wegovy preferred (no step)</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Not documented</t>
+          <t>12</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Not documented</t>
+          <t>Quantity per 30 days (no numeric limit on form); renewal requires 5% weight loss (adults) or 4% BMI reduction (adolescents)</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>NC Medicaid PDL applies to FFS and Standard Plans</t>
+          <t>NC Medicaid PA form for GLP-1s for weight management (Carolina Complete Health, version 202407), applies across FFS and Standard Plans</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>8/1/2024</t>
+          <t>7/1/2024</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>NC Medicaid PDL revised 8.1.2024 (p. 31); NC Medicaid PA request form for GLP-1s Wegovy and Zepbound (2025 version)</t>
+          <t>NC Medicaid Pharmacy Prior Approval Request for GLP-1s for Weight Management, version 202407, https://network.carolinacompletehealth.com/content/dam/centene/carolinacompletehealth/pdfs/CCH_GLP-1_Weight_Management_Request_Form.pdf</t>
         </is>
       </c>
     </row>
@@ -7022,47 +7022,47 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>fda_label (per Klebanoff); criteria not in documents in hand</t>
+          <t>more_restrictive (MCO form; requires concurrent diabetes or antidiabetic use in past 120 days before a preferred GLP-1)</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Not in documents in hand (PDL marks PA, QL)</t>
+          <t>Age 18 or older: BMI 30 or higher, or 27 to under 30 with at least one comorbidity (CVD, dyslipidemia, hypertension, metabolic syndrome, OSA, prediabetes, type 2 diabetes)</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Not documented</t>
+          <t>Under 18: BMI at or above the 95th percentile standardized for age and sex (current CDC charts)</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>None documented (Saxenda, Wegovy, Zepbound all preferred)</t>
+          <t>Preferred GLP-1 for obesity requires a concurrent diabetes diagnosis OR an antidiabetic drug in the past 120 days with trial/failure, contraindication or intolerance to Ozempic, Trulicity or Victoza; non-preferred requires trial/failure of the preferred obesity agents and preferred hypoglycemics</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Not documented</t>
+          <t>18 (adult); 12 to 17 covered under adolescent criteria</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>QL flagged on PDL; detail not in documents in hand</t>
+          <t>Quantity limits per the PA Health &amp; Wellness website (not on the form)</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Statewide PDL (FFS and MCOs)</t>
+          <t>PA Health &amp; Wellness (Centene MCO) Obesity Treatment Agents PA form, effective 1/6/2025; statewide FFS criteria (Klebanoff June 2024) coded PA at FDA label</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>7/7/2025</t>
+          <t>1/6/2025</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>Pennsylvania Statewide PDL January 9, 2023 (p. 40); January 8, 2024 (p. 41); July 7, 2025 (p. 43)</t>
+          <t>PA Health &amp; Wellness Obesity Treatment Agents Prior Authorization Form, effective 1/6/2025, https://pahealthwellness.com/content/dam/centene/Pennsylvania/policies/FaxFormsMedication/Obesity%20Treatment%20Agents%20Fax%20Form%20v1.2025.pdf</t>
         </is>
       </c>
     </row>
@@ -7074,47 +7074,47 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>not_documented (clinical PA for entire class, manual PA)</t>
+          <t>more_restrictive (6-month supervised weight-management program before drug therapy; MCO policy)</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Not in FFS documents in hand. Neighborhood Health Plan of RI (Medicaid MCO) Weight Loss Management policy (eff. 7/2018, reviewed through 08/2023): BMI 30 or higher, or 27 or higher with a risk factor; 6 months of a comprehensive weight management program before drug therapy; Saxenda requires inadequate response to Contrave or Wegovy</t>
+          <t>Adults: BMI 30 or higher, or 27 or higher with at least one risk factor (coronary heart disease, type 2 diabetes, dyslipidemia, hypertension, sleep apnea); Wegovy MACE pathway: BMI 27 or higher with established CVD and no type 2 diabetes</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>MCO policy: age 12 and older with BMI classified obese for age and sex</t>
+          <t>Ages 12 and older: BMI 30 or higher, or BMI classified as obese standardized for age and sex (Wegovy)</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>FFS: not documented; MCO policy: Saxenda after Contrave or Wegovy</t>
+          <t>Comprehensive weight-management program with behavioral counseling, nutrition and activity, monthly meetings for at least 6 months before drug therapy; prescribed by or with a weight-loss clinic or dietitian; no concurrent GLP-1</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>12 (MCO policy)</t>
+          <t>12 (Wegovy); 18 (Zepbound, Contrave)</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Not documented (evidence file: QL No)</t>
+          <t>Wegovy and Zepbound 4 pens per 28 days; initial and continuation 6 months each; continuation requires 5% baseline weight loss at the maintenance dose</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>FFS PDL; MCO (Neighborhood) policy differs</t>
+          <t>Neighborhood Health Plan of RI (Medicaid MCO) policy; FFS PDL applies a manual clinical PA to the whole class</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>5/21/2024</t>
+          <t>5/15/2024</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>RI EOHHS FFS PDL January 10, 2023 (p. 45) and October 1, 2024 (p. 42); Neighborhood Health Plan of RI, Weight Loss Management policy, reviewed 08/2023</t>
+          <t>Neighborhood Health Plan of RI, Weight Loss Management policy (Scope: Medicaid), effective 7/2018, reviewed through 5/2024, https://www.nhpri.org/wp-content/uploads/2024/08/Medicaid_Weight_Loss_Contrave_Wegovy_Zepbound_20240515_aCAS.pdf; RI EOHHS FFS PDL (manual PA, review date 5/21/2024)</t>
         </is>
       </c>
     </row>
@@ -7174,37 +7174,37 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>not_documented (PA, QL flagged; criteria in Optum Rx TennCare criteria document, not in folder)</t>
+          <t>fda_label</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Not in documents in hand</t>
+          <t>Adults: BMI 30 or higher, or 27 or higher with a weight-related comorbidity (hypertension, dyslipidemia, diabetes, coronary heart disease, MASH/NASH, OSA)</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Not documented</t>
+          <t>Under 18 (Wegovy, Saxenda): BMI at or above the 95th percentile standardized for age and sex</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Not documented</t>
+          <t>Wegovy and Zepbound preferred (no step); Saxenda non-preferred (trial and failure, contraindication or intolerance to two preferred agents)</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Not documented</t>
+          <t>12 (Wegovy, Saxenda); 18 (Zepbound)</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>QL flagged on PDL</t>
+          <t>Wegovy and Zepbound 4 injections per month; Saxenda 3 mg/day; renewal requires 5% weight loss (one-month bridge if not met)</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>TennCare PDL (MCOs via Optum Rx)</t>
+          <t>TennCare (MCOs via Optum Rx)</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
@@ -7214,7 +7214,7 @@
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>TennCare PDL effective August 1, 2025 (p. 23); SPA TN-25-0006</t>
+          <t>TennCare Pharmacy Program Provider Notice, Obesity Management Agents, effective August 1, 2025, https://contenthub-aem.optumrx.com/content/dam/contenthub/onboarding/assets/Tenncare/Provider-Notice-Obesity-Management-Agents-08-01-25.pdf</t>
         </is>
       </c>
     </row>
@@ -7226,37 +7226,37 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>not_documented (PA criteria document on Utah Medicaid PA page, not in folder)</t>
+          <t>more_restrictive (6 months of dietitian-supervised lifestyle trials required)</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Not in documents in hand</t>
+          <t>Adults: BMI 30 or higher (obesity), or 27 to 29.9 with at least one weight-related comorbidity (hypertension, dyslipidemia)</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Not documented</t>
+          <t>Under 18 (Saxenda, Wegovy): BMI at or above the 95th percentile for age and sex</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Not documented</t>
+          <t>At least 6 months of strict lifestyle interventions (dietitian-prescribed reduced-calorie diet, aerobic and resistance exercise) without reaching 5% weight loss; not concurrently on another GLP-1; must not have type 2 diabetes, OSA or MACE (separate forms for those)</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Not documented</t>
+          <t>12 (Saxenda, Wegovy); 18 (Zepbound)</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Not documented</t>
+          <t>Initial and renewal up to 6 months each; Saxenda discontinued if under 4% loss at week 16 (adults); renewal requires 5% weight loss and continued dietitian follow-up</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>Utah Medicaid PDL (FFS; ACOs follow)</t>
+          <t>Utah Medicaid FFS PA form (ACOs follow)</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
@@ -7266,7 +7266,7 @@
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>Utah Medicaid PDL and resources effective August 1, 2025, PA criteria table: GLP-1 Medications for Weight Loss, Saxenda, Wegovy, Zepbound, 07/01/25</t>
+          <t>Utah Medicaid Pharmacy Prior Authorization Request Form, GLP-1 Medications for Weight Loss (Saxenda, Wegovy, Zepbound), last updated 7-1-25, https://medicaid-documents.dhhs.utah.gov/pharmacy/priorauthorization/pdf/GLP-1%20Medications%20for%20Weight%20Loss%20(Saxenda,%20Wegovy,%20Zepbound).pdf</t>
         </is>
       </c>
     </row>

</xml_diff>